<commit_message>
fix(ai): fix ISPU calculation
</commit_message>
<xml_diff>
--- a/reports/ispu_future.xlsx
+++ b/reports/ispu_future.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,9 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -425,161 +431,1131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>pollutant</t>
+          <t>y1_ispu_tft_pred</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ISPU_tft</t>
+          <t>y1_ispu_nbeats_pred</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>category_ISPU_tft</t>
+          <t>y2_ispu_tft_pred</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ISPU_nbeats</t>
+          <t>y2_ispu_nbeats_pred</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>category_ISPU_nbeats</t>
+          <t>y3_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>y3_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>y4_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>y4_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>y5_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>y5_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>y1_category_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>y1_category_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>y2_category_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>y2_category_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>y3_category_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>y3_category_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>y4_category_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>y4_category_ispu_nbeats_pred</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>y5_category_ispu_tft_pred</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>y5_category_ispu_nbeats_pred</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>y1</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B2" t="n">
+        <v>60</v>
       </c>
       <c r="C2" t="n">
-        <v>56</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sedang</t>
-        </is>
+        <v>67</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>58</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Sedang</t>
+        <v>34</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H2" t="n">
+        <v>17</v>
+      </c>
+      <c r="I2" t="n">
+        <v>19</v>
+      </c>
+      <c r="J2" t="n">
+        <v>14</v>
+      </c>
+      <c r="K2" t="n">
+        <v>11</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Baik</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>y2</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>45839.04166666666</v>
+      </c>
+      <c r="B3" t="n">
+        <v>60</v>
       </c>
       <c r="C3" t="n">
-        <v>28</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Baik</t>
-        </is>
+        <v>66</v>
+      </c>
+      <c r="D3" t="n">
+        <v>31</v>
       </c>
       <c r="E3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F3" t="inlineStr">
+        <v>32</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I3" t="n">
+        <v>18</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>Baik</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>y3</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>45839.08333333334</v>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
       </c>
       <c r="C4" t="n">
+        <v>64</v>
+      </c>
+      <c r="D4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" t="n">
         <v>10</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Baik</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Baik</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>y4</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>45839.125</v>
+      </c>
+      <c r="B5" t="n">
+        <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Baik</t>
-        </is>
+        <v>62</v>
+      </c>
+      <c r="D5" t="n">
+        <v>31</v>
       </c>
       <c r="E5" t="n">
+        <v>29</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>16</v>
+      </c>
+      <c r="I5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J5" t="n">
         <v>14</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="K5" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Baik</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>y5</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>45839.16666666666</v>
+      </c>
+      <c r="B6" t="n">
+        <v>59</v>
       </c>
       <c r="C6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E6" t="n">
+        <v>28</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" t="n">
         <v>16</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Baik</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>45839.20833333334</v>
+      </c>
+      <c r="B7" t="n">
+        <v>58</v>
+      </c>
+      <c r="C7" t="n">
+        <v>59</v>
+      </c>
+      <c r="D7" t="n">
+        <v>31</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" t="n">
+        <v>16</v>
+      </c>
+      <c r="J7" t="n">
+        <v>15</v>
+      </c>
+      <c r="K7" t="n">
+        <v>11</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>45839.25</v>
+      </c>
+      <c r="B8" t="n">
+        <v>57</v>
+      </c>
+      <c r="C8" t="n">
+        <v>58</v>
+      </c>
+      <c r="D8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E8" t="n">
+        <v>27</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" t="n">
+        <v>16</v>
+      </c>
+      <c r="K8" t="n">
+        <v>11</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>45839.29166666666</v>
+      </c>
+      <c r="B9" t="n">
+        <v>57</v>
+      </c>
+      <c r="C9" t="n">
+        <v>57</v>
+      </c>
+      <c r="D9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" t="n">
+        <v>28</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>14</v>
+      </c>
+      <c r="I9" t="n">
+        <v>14</v>
+      </c>
+      <c r="J9" t="n">
+        <v>16</v>
+      </c>
+      <c r="K9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>45839.33333333334</v>
+      </c>
+      <c r="B10" t="n">
+        <v>56</v>
+      </c>
+      <c r="C10" t="n">
+        <v>58</v>
+      </c>
+      <c r="D10" t="n">
+        <v>28</v>
+      </c>
+      <c r="E10" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13</v>
+      </c>
+      <c r="I10" t="n">
+        <v>14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>16</v>
+      </c>
+      <c r="K10" t="n">
+        <v>11</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45839.375</v>
+      </c>
+      <c r="B11" t="n">
+        <v>56</v>
+      </c>
+      <c r="C11" t="n">
+        <v>58</v>
+      </c>
+      <c r="D11" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" t="n">
+        <v>28</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" t="n">
+        <v>13</v>
+      </c>
+      <c r="I11" t="n">
+        <v>14</v>
+      </c>
+      <c r="J11" t="n">
+        <v>15</v>
+      </c>
+      <c r="K11" t="n">
+        <v>11</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45839.41666666666</v>
+      </c>
+      <c r="B12" t="n">
+        <v>56</v>
+      </c>
+      <c r="C12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D12" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" t="n">
+        <v>28</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" t="n">
+        <v>13</v>
+      </c>
+      <c r="I12" t="n">
+        <v>14</v>
+      </c>
+      <c r="J12" t="n">
+        <v>15</v>
+      </c>
+      <c r="K12" t="n">
+        <v>10</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>45839.45833333334</v>
+      </c>
+      <c r="B13" t="n">
+        <v>56</v>
+      </c>
+      <c r="C13" t="n">
+        <v>58</v>
+      </c>
+      <c r="D13" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" t="n">
+        <v>28</v>
+      </c>
+      <c r="F13" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" t="n">
+        <v>9</v>
+      </c>
+      <c r="H13" t="n">
+        <v>13</v>
+      </c>
+      <c r="I13" t="n">
+        <v>14</v>
+      </c>
+      <c r="J13" t="n">
+        <v>15</v>
+      </c>
+      <c r="K13" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Sedang</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Baik</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
         <is>
           <t>Baik</t>
         </is>

</xml_diff>